<commit_message>
20260416 log and analysis #13
</commit_message>
<xml_diff>
--- a/test/Analysis.xlsx
+++ b/test/Analysis.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="12200"/>
+    <workbookView windowWidth="24750" windowHeight="12200" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="2026-04-15" sheetId="1" r:id="rId1"/>
+    <sheet name="2026-04-16" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1797" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2184" uniqueCount="137">
   <si>
     <t>TaskID</t>
   </si>
@@ -1053,8 +1054,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1677,7 +1681,6 @@
       <c r="E3">
         <v>60.99</v>
       </c>
-      <c r="F3"/>
       <c r="I3" t="s">
         <v>14</v>
       </c>
@@ -1710,7 +1713,6 @@
       <c r="E4">
         <v>49.96</v>
       </c>
-      <c r="F4"/>
       <c r="I4" t="s">
         <v>16</v>
       </c>
@@ -13475,6 +13477,2608 @@
         <v>1047.267</v>
       </c>
       <c r="F595">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:L125"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14"/>
+  <cols>
+    <col min="9" max="9" width="15.1818181818182" customWidth="1"/>
+    <col min="10" max="10" width="18.5454545454545" customWidth="1"/>
+    <col min="11" max="11" width="15.1818181818182" customWidth="1"/>
+    <col min="12" max="12" width="10.5454545454545" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1">
+        <v>4674</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="1">
+        <v>26.797</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K2" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L2" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="1">
+        <v>4006</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="1">
+        <v>7.472</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3">
+        <f>AVERAGE(E2:E17)</f>
+        <v>10.968875</v>
+      </c>
+      <c r="K3">
+        <f>MAX(E2:E17)</f>
+        <v>48.336</v>
+      </c>
+      <c r="L3">
+        <f>_xlfn.PERCENTILE.INC(E2:E17,0.9)</f>
+        <v>28.6375</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="1">
+        <v>4008</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" s="1">
+        <v>2.647</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4">
+        <f>AVERAGE(E104:E125)</f>
+        <v>1153.56795454545</v>
+      </c>
+      <c r="K4">
+        <f>MAX(E104:E125)</f>
+        <v>5512.169</v>
+      </c>
+      <c r="L4">
+        <f>_xlfn.PERCENTILE.INC(E104:E125,0.9)</f>
+        <v>1841.4607</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="1">
+        <v>4010</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="1">
+        <v>6.022</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5">
+        <f>AVERAGE(E38:E103)</f>
+        <v>64.4157575757576</v>
+      </c>
+      <c r="K5">
+        <f>MAX(E38:E103)</f>
+        <v>72.281</v>
+      </c>
+      <c r="L5">
+        <f>_xlfn.PERCENTILE.INC(E38:E103,0.9)</f>
+        <v>67.7795</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="1">
+        <v>4011</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.909</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6">
+        <f>AVERAGE(E18:E37)</f>
+        <v>260.5569</v>
+      </c>
+      <c r="K6">
+        <f>MAX(E18:E37)</f>
+        <v>2787.006</v>
+      </c>
+      <c r="L6">
+        <f>_xlfn.PERCENTILE.INC(E18:E37,0.9)</f>
+        <v>425.193900000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="1">
+        <v>4012</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="1">
+        <v>8.279</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="1">
+        <v>4013</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="1">
+        <v>2.83</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="1">
+        <v>4014</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1.549</v>
+      </c>
+      <c r="F9" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" s="1">
+        <v>4015</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="1">
+        <v>1.523</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" s="1">
+        <v>4009</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="1">
+        <v>1.113</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" s="1">
+        <v>4603</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="1">
+        <v>5.986</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" s="1">
+        <v>4005</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E13" s="1">
+        <v>2.79</v>
+      </c>
+      <c r="F13" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" s="1">
+        <v>4007</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" s="1">
+        <v>3.799</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" s="1">
+        <v>4688</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="1">
+        <v>30.478</v>
+      </c>
+      <c r="F15" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" s="1">
+        <v>4704</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="1">
+        <v>24.972</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="1">
+        <v>4820</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="1">
+        <v>48.336</v>
+      </c>
+      <c r="F17" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="1">
+        <v>3008</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" s="1">
+        <v>210.361</v>
+      </c>
+      <c r="F18" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="1">
+        <v>3009</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" s="1">
+        <v>81.106</v>
+      </c>
+      <c r="F19" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="1">
+        <v>3010</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="1">
+        <v>378.99</v>
+      </c>
+      <c r="F20" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="1">
+        <v>3011</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="1">
+        <v>2787.006</v>
+      </c>
+      <c r="F21" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="1">
+        <v>3012</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="1">
+        <v>61.737</v>
+      </c>
+      <c r="F22" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="1">
+        <v>3013</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E23" s="1">
+        <v>62.43</v>
+      </c>
+      <c r="F23" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="1">
+        <v>3014</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E24" s="1">
+        <v>70.703</v>
+      </c>
+      <c r="F24" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="1">
+        <v>3015</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="1">
+        <v>62.875</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="1">
+        <v>3000</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26" s="1">
+        <v>49.132</v>
+      </c>
+      <c r="F26" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="1">
+        <v>3000</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E27" s="1">
+        <v>841.029</v>
+      </c>
+      <c r="F27" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="1">
+        <v>3001</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E28" s="1">
+        <v>105.446</v>
+      </c>
+      <c r="F28" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="1">
+        <v>3002</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E29" s="1">
+        <v>52.609</v>
+      </c>
+      <c r="F29" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="1">
+        <v>3003</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E30" s="1">
+        <v>56.261</v>
+      </c>
+      <c r="F30" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="1">
+        <v>3004</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E31" s="1">
+        <v>52.418</v>
+      </c>
+      <c r="F31" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="1">
+        <v>3005</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="1">
+        <v>54.702</v>
+      </c>
+      <c r="F32" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="1">
+        <v>3006</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" s="1">
+        <v>53.54</v>
+      </c>
+      <c r="F33" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="1">
+        <v>3007</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E34" s="1">
+        <v>66.392</v>
+      </c>
+      <c r="F34" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="1">
+        <v>3008</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E35" s="1">
+        <v>52.227</v>
+      </c>
+      <c r="F35" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="1">
+        <v>3009</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E36" s="1">
+        <v>60.945</v>
+      </c>
+      <c r="F36" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="1">
+        <v>3010</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E37" s="1">
+        <v>51.229</v>
+      </c>
+      <c r="F37" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="1">
+        <v>0</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E38" s="1">
+        <v>65.971</v>
+      </c>
+      <c r="F38" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="1">
+        <v>1</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E39" s="1">
+        <v>62.136</v>
+      </c>
+      <c r="F39" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="1">
+        <v>2</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E40" s="1">
+        <v>65.816</v>
+      </c>
+      <c r="F40" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="1">
+        <v>3</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E41" s="1">
+        <v>72.281</v>
+      </c>
+      <c r="F41" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="1">
+        <v>4</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E42" s="1">
+        <v>62.38</v>
+      </c>
+      <c r="F42" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="1">
+        <v>5</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E43" s="1">
+        <v>67.374</v>
+      </c>
+      <c r="F43" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="1">
+        <v>6</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E44" s="1">
+        <v>64.721</v>
+      </c>
+      <c r="F44" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="1">
+        <v>7</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E45" s="1">
+        <v>62.033</v>
+      </c>
+      <c r="F45" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="1">
+        <v>8</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E46" s="1">
+        <v>62.199</v>
+      </c>
+      <c r="F46" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="1">
+        <v>9</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E47" s="1">
+        <v>66.491</v>
+      </c>
+      <c r="F47" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="1">
+        <v>10</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E48" s="1">
+        <v>62.067</v>
+      </c>
+      <c r="F48" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="1">
+        <v>11</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E49" s="1">
+        <v>69.358</v>
+      </c>
+      <c r="F49" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" s="1">
+        <v>12</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E50" s="1">
+        <v>64.011</v>
+      </c>
+      <c r="F50" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="1">
+        <v>13</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E51" s="1">
+        <v>65.305</v>
+      </c>
+      <c r="F51" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="1">
+        <v>14</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E52" s="1">
+        <v>65.872</v>
+      </c>
+      <c r="F52" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="1">
+        <v>15</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E53" s="1">
+        <v>68.185</v>
+      </c>
+      <c r="F53" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="1">
+        <v>16</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E54" s="1">
+        <v>68.562</v>
+      </c>
+      <c r="F54" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="1">
+        <v>17</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E55" s="1">
+        <v>64.094</v>
+      </c>
+      <c r="F55" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="1">
+        <v>18</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E56" s="1">
+        <v>62.037</v>
+      </c>
+      <c r="F56" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" s="1">
+        <v>19</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E57" s="1">
+        <v>64.896</v>
+      </c>
+      <c r="F57" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" s="1">
+        <v>20</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E58" s="1">
+        <v>64.982</v>
+      </c>
+      <c r="F58" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" s="1">
+        <v>21</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E59" s="1">
+        <v>65.454</v>
+      </c>
+      <c r="F59" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" s="1">
+        <v>22</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E60" s="1">
+        <v>62.173</v>
+      </c>
+      <c r="F60" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" s="1">
+        <v>23</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E61" s="1">
+        <v>62.402</v>
+      </c>
+      <c r="F61" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" s="1">
+        <v>24</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E62" s="1">
+        <v>66.343</v>
+      </c>
+      <c r="F62" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" s="1">
+        <v>25</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E63" s="1">
+        <v>64.036</v>
+      </c>
+      <c r="F63" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" s="1">
+        <v>26</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E64" s="1">
+        <v>62.139</v>
+      </c>
+      <c r="F64" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="1">
+        <v>27</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E65" s="1">
+        <v>63.711</v>
+      </c>
+      <c r="F65" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" s="1">
+        <v>28</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E66" s="1">
+        <v>62.273</v>
+      </c>
+      <c r="F66" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" s="1">
+        <v>29</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E67" s="1">
+        <v>62.151</v>
+      </c>
+      <c r="F67" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" s="1">
+        <v>30</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E68" s="1">
+        <v>62.169</v>
+      </c>
+      <c r="F68" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" s="1">
+        <v>31</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E69" s="1">
+        <v>62.257</v>
+      </c>
+      <c r="F69" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" s="1">
+        <v>32</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E70" s="1">
+        <v>65.762</v>
+      </c>
+      <c r="F70" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" s="1">
+        <v>33</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E71" s="1">
+        <v>62.167</v>
+      </c>
+      <c r="F71" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" s="1">
+        <v>34</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E72" s="1">
+        <v>62.126</v>
+      </c>
+      <c r="F72" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" s="1">
+        <v>35</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E73" s="1">
+        <v>62.055</v>
+      </c>
+      <c r="F73" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" s="1">
+        <v>36</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E74" s="1">
+        <v>62.473</v>
+      </c>
+      <c r="F74" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="A75" s="1">
+        <v>37</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E75" s="1">
+        <v>62.052</v>
+      </c>
+      <c r="F75" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" s="1">
+        <v>38</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E76" s="1">
+        <v>65.586</v>
+      </c>
+      <c r="F76" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" s="1">
+        <v>39</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E77" s="1">
+        <v>63.188</v>
+      </c>
+      <c r="F77" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="A78" s="1">
+        <v>40</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E78" s="1">
+        <v>65.269</v>
+      </c>
+      <c r="F78" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="A79" s="1">
+        <v>41</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E79" s="1">
+        <v>63.46</v>
+      </c>
+      <c r="F79" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="A80" s="1">
+        <v>42</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E80" s="1">
+        <v>62.055</v>
+      </c>
+      <c r="F80" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
+      <c r="A81" s="1">
+        <v>43</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E81" s="1">
+        <v>66.292</v>
+      </c>
+      <c r="F81" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6">
+      <c r="A82" s="1">
+        <v>44</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E82" s="1">
+        <v>62.872</v>
+      </c>
+      <c r="F82" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6">
+      <c r="A83" s="1">
+        <v>45</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E83" s="1">
+        <v>68.885</v>
+      </c>
+      <c r="F83" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6">
+      <c r="A84" s="1">
+        <v>46</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E84" s="1">
+        <v>63.718</v>
+      </c>
+      <c r="F84" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
+      <c r="A85" s="1">
+        <v>47</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E85" s="1">
+        <v>67.347</v>
+      </c>
+      <c r="F85" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6">
+      <c r="A86" s="1">
+        <v>48</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E86" s="1">
+        <v>71.825</v>
+      </c>
+      <c r="F86" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6">
+      <c r="A87" s="1">
+        <v>49</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E87" s="1">
+        <v>63.104</v>
+      </c>
+      <c r="F87" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6">
+      <c r="A88" s="1">
+        <v>50</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E88" s="1">
+        <v>62.054</v>
+      </c>
+      <c r="F88" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6">
+      <c r="A89" s="1">
+        <v>51</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E89" s="1">
+        <v>62.179</v>
+      </c>
+      <c r="F89" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6">
+      <c r="A90" s="1">
+        <v>52</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E90" s="1">
+        <v>62.245</v>
+      </c>
+      <c r="F90" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6">
+      <c r="A91" s="1">
+        <v>53</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E91" s="1">
+        <v>70.1</v>
+      </c>
+      <c r="F91" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6">
+      <c r="A92" s="1">
+        <v>54</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E92" s="1">
+        <v>62.128</v>
+      </c>
+      <c r="F92" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
+      <c r="A93" s="1">
+        <v>55</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E93" s="1">
+        <v>65.374</v>
+      </c>
+      <c r="F93" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" s="1">
+        <v>56</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E94" s="1">
+        <v>62.206</v>
+      </c>
+      <c r="F94" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
+      <c r="A95" s="1">
+        <v>57</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E95" s="1">
+        <v>64.234</v>
+      </c>
+      <c r="F95" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6">
+      <c r="A96" s="1">
+        <v>58</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E96" s="1">
+        <v>64.342</v>
+      </c>
+      <c r="F96" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6">
+      <c r="A97" s="1">
+        <v>59</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E97" s="1">
+        <v>66.682</v>
+      </c>
+      <c r="F97" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6">
+      <c r="A98" s="1">
+        <v>60</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E98" s="1">
+        <v>65.382</v>
+      </c>
+      <c r="F98" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6">
+      <c r="A99" s="1">
+        <v>61</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E99" s="1">
+        <v>66.926</v>
+      </c>
+      <c r="F99" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6">
+      <c r="A100" s="1">
+        <v>62</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E100" s="1">
+        <v>62.094</v>
+      </c>
+      <c r="F100" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6">
+      <c r="A101" s="1">
+        <v>63</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E101" s="1">
+        <v>64.518</v>
+      </c>
+      <c r="F101" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6">
+      <c r="A102" s="1">
+        <v>64</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E102" s="1">
+        <v>62.051</v>
+      </c>
+      <c r="F102" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6">
+      <c r="A103" s="1">
+        <v>65</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E103" s="1">
+        <v>62.81</v>
+      </c>
+      <c r="F103" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6">
+      <c r="A104" s="1">
+        <v>2013</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E104" s="1">
+        <v>827.722</v>
+      </c>
+      <c r="F104" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6">
+      <c r="A105" s="1">
+        <v>2014</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E105" s="1">
+        <v>832.024</v>
+      </c>
+      <c r="F105" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6">
+      <c r="A106" s="1">
+        <v>2015</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E106" s="1">
+        <v>765.971</v>
+      </c>
+      <c r="F106" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6">
+      <c r="A107" s="1">
+        <v>2016</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E107" s="1">
+        <v>1894.486</v>
+      </c>
+      <c r="F107" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6">
+      <c r="A108" s="1">
+        <v>2017</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E108" s="1">
+        <v>679.751</v>
+      </c>
+      <c r="F108" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6">
+      <c r="A109" s="1">
+        <v>2018</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E109" s="1">
+        <v>760.571</v>
+      </c>
+      <c r="F109" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6">
+      <c r="A110" s="1">
+        <v>2019</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E110" s="1">
+        <v>1312.868</v>
+      </c>
+      <c r="F110" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6">
+      <c r="A111" s="1">
+        <v>2020</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E111" s="1">
+        <v>1364.233</v>
+      </c>
+      <c r="F111" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6">
+      <c r="A112" s="1">
+        <v>2000</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E112" s="1">
+        <v>1035.744</v>
+      </c>
+      <c r="F112" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6">
+      <c r="A113" s="1">
+        <v>2000</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E113" s="1">
+        <v>5512.169</v>
+      </c>
+      <c r="F113" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6">
+      <c r="A114" s="1">
+        <v>2001</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E114" s="1">
+        <v>2663.948</v>
+      </c>
+      <c r="F114" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6">
+      <c r="A115" s="1">
+        <v>2002</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E115" s="1">
+        <v>707.737</v>
+      </c>
+      <c r="F115" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6">
+      <c r="A116" s="1">
+        <v>2003</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E116" s="1">
+        <v>715.369</v>
+      </c>
+      <c r="F116" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6">
+      <c r="A117" s="1">
+        <v>2004</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E117" s="1">
+        <v>711.649</v>
+      </c>
+      <c r="F117" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6">
+      <c r="A118" s="1">
+        <v>2005</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E118" s="1">
+        <v>692.597</v>
+      </c>
+      <c r="F118" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6">
+      <c r="A119" s="1">
+        <v>2006</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D119" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E119" s="1">
+        <v>717.328</v>
+      </c>
+      <c r="F119" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6">
+      <c r="A120" s="1">
+        <v>2007</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E120" s="1">
+        <v>707.235</v>
+      </c>
+      <c r="F120" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6">
+      <c r="A121" s="1">
+        <v>2008</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E121" s="1">
+        <v>649.134</v>
+      </c>
+      <c r="F121" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6">
+      <c r="A122" s="1">
+        <v>2009</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E122" s="1">
+        <v>727.932</v>
+      </c>
+      <c r="F122" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6">
+      <c r="A123" s="1">
+        <v>2010</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E123" s="1">
+        <v>695.369</v>
+      </c>
+      <c r="F123" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6">
+      <c r="A124" s="1">
+        <v>2011</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E124" s="1">
+        <v>706.91</v>
+      </c>
+      <c r="F124" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6">
+      <c r="A125" s="1">
+        <v>2012</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E125" s="1">
+        <v>697.748</v>
+      </c>
+      <c r="F125" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>